<commit_message>
Fix backend database connection handling
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1583,6 +1583,70 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>36.891, 10.172</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F22" t="n">
+        <v>22</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>blob:http://localhost:8081/9514252d-d269-4104-801b-cc6ef0d05b9a</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix owner notifications, sync property occupancy, and load real owner applications
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1711,6 +1711,70 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>36.892, 10.188</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>19</v>
+      </c>
+      <c r="F24" t="n">
+        <v>22</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775208903/dhg8vzea1ivxdammgoyz.png</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>relaxed</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>rarely</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Theme + language updates
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1775,6 +1775,534 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>36.891, 10.172</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>22</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775418008/dwqf3swmezih8gabavdv.jpg</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>relaxed</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>rarely</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>22</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775418300/iighfa0dsqhmnyrqolfj.jpg</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>relaxed</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>quiet</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>rarely</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>46</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775423081/zljyqidmevq6zk2huidn.png</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>relaxed</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>quiet</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>rarely</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>8</v>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>46</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775423081/zljyqidmevq6zk2huidn.png</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>8</v>
+      </c>
+      <c r="B29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>46</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775423081/zljyqidmevq6zk2huidn.png</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>8</v>
+      </c>
+      <c r="B30" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>46</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775423081/zljyqidmevq6zk2huidn.png</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>46</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775423081/zljyqidmevq6zk2huidn.png</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>36.891, 10.172</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>16</v>
+      </c>
+      <c r="F32" t="n">
+        <v>24</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>STUDENT</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775424522/cpcsr7hklqpb0qhs3mev.jpg</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>quiet</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>10</v>
+      </c>
+      <c r="B33" t="n">
+        <v>9</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>36.891, 10.172</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>16</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>STUDENT</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dajunvjml/image/upload/v1775424522/cpcsr7hklqpb0qhs3mev.jpg</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Change seeker selection to radio buttons
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2303,6 +2303,134 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>12</v>
+      </c>
+      <c r="B34" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>36.892, 10.187</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>23</v>
+      </c>
+      <c r="F34" t="n">
+        <v>38</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775469266/iva8ka4cytun63zywnyp.jpg</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>rarely</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B35" t="n">
+        <v>16</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>36.892, 10.188</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" t="n">
+        <v>22</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775556566/j39en7kkx9gbex03h426.jpg</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>quiet</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajout du modèle IA et script de génération de données
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2431,6 +2431,262 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>15</v>
+      </c>
+      <c r="B36" t="n">
+        <v>17</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>roommate</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>36.892, 10.187</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>23</v>
+      </c>
+      <c r="F36" t="n">
+        <v>18</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775559731/sshzueba5ki8uikn5uo2.jpg</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>16</v>
+      </c>
+      <c r="B37" t="n">
+        <v>18</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>36.892, 10.188</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>10</v>
+      </c>
+      <c r="F37" t="n">
+        <v>17</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775559851/xz7j9c4ko7zkfx8dhybk.webp</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>relaxed</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>17</v>
+      </c>
+      <c r="B38" t="n">
+        <v>19</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>36.892, 10.187</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>10</v>
+      </c>
+      <c r="F38" t="n">
+        <v>38</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775560356/x13n4pm7mnzxejwpnkar.jpg</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B39" t="n">
+        <v>20</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>36.892, 10.187</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>10</v>
+      </c>
+      <c r="F39" t="n">
+        <v>40</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775560461/vd7bkjfjn80j0ry24i8a.jpg</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>tidy</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>quiet</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>often</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update AI property matching, filtering, and UI components
</commit_message>
<xml_diff>
--- a/backend/seeker_profiles.xlsx
+++ b/backend/seeker_profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2687,6 +2687,80 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>30</v>
+      </c>
+      <c r="B40" t="n">
+        <v>23</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>36.683, 10.161</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>23</v>
+      </c>
+      <c r="F40" t="n">
+        <v>23</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/doictcopf/image/upload/v1775855589/akm6hswryghzwpwsqsg4.png</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>sleepy girl</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>very clean and well organized girl</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i have a lot of friends </t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>not much</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>hard working girl</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sports healthy lifestyles reading books </t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>respect</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>